<commit_message>
marked fields to get from biotics
</commit_message>
<xml_diff>
--- a/docs/iNat-to-Obs.xlsx
+++ b/docs/iNat-to-Obs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lwise\Documents\iNaturalist\ObsXwalk\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Syd\Documents\INR\iNatDataPipeline\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B38E29-5792-4A81-9B22-8D3A0BBF995D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCDA347-9F56-4D8A-937B-0F3BC119FCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8925" yWindow="0" windowWidth="28800" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="iNatObsXwalk" sheetId="2" r:id="rId1"/>
@@ -18,16 +18,11 @@
     <sheet name="species" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="354">
   <si>
     <t>id</t>
   </si>
@@ -1086,6 +1081,9 @@
   </si>
   <si>
     <t>use to populate all other Biotics element fields</t>
+  </si>
+  <si>
+    <t>from biotics</t>
   </si>
 </sst>
 </file>
@@ -1669,9 +1667,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1709,7 +1707,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1815,7 +1813,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1957,7 +1955,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2408,7 +2406,7 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C47" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D47" s="4" t="s">
         <v>69</v>
@@ -2416,7 +2414,7 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C48" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D48" s="4" t="s">
         <v>71</v>
@@ -2424,7 +2422,7 @@
     </row>
     <row r="49" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C49" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D49" s="4" t="s">
         <v>36</v>
@@ -2435,7 +2433,7 @@
     </row>
     <row r="50" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C50" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>37</v>
@@ -2443,7 +2441,7 @@
     </row>
     <row r="51" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D51" s="4" t="s">
         <v>75</v>
@@ -2451,7 +2449,7 @@
     </row>
     <row r="52" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C52" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D52" s="4" t="s">
         <v>77</v>
@@ -2459,7 +2457,7 @@
     </row>
     <row r="53" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C53" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D53" s="4" t="s">
         <v>79</v>
@@ -2467,7 +2465,7 @@
     </row>
     <row r="54" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C54" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>81</v>
@@ -2475,7 +2473,7 @@
     </row>
     <row r="55" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C55" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D55" s="4" t="s">
         <v>84</v>
@@ -2483,7 +2481,7 @@
     </row>
     <row r="56" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C56" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D56" s="4" t="s">
         <v>86</v>

</xml_diff>